<commit_message>
feat: dual-header Excel template for HR import
- template_import.xlsx: row 1 = Chinese guide, row 2 = English
  column names, row 3+ = data. HR reads Chinese, system parses
  English, no separate reference doc needed.
- ona_import.py: skiprows=1 so backend skips Chinese guide row
  and reads English column names + data from row 2 onward.
- data_import_spec.md, import_field_mapping.md: updated to
  document the dual-header structure.

Co-Authored-By: Claude Haiku 4.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/frontend/public/template_import.xlsx
+++ b/frontend/public/template_import.xlsx
@@ -14,102 +14,156 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="50">
+  <si>
+    <t>年龄</t>
+  </si>
   <si>
     <t>Age</t>
   </si>
   <si>
+    <t>状态</t>
+  </si>
+  <si>
     <t>Attrition</t>
   </si>
   <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>出差频率</t>
+  </si>
+  <si>
     <t>BusinessTravel</t>
   </si>
   <si>
+    <t>Travel_Frequently</t>
+  </si>
+  <si>
+    <t>Travel_Rarely</t>
+  </si>
+  <si>
+    <t>部门</t>
+  </si>
+  <si>
     <t>Department</t>
   </si>
   <si>
+    <t>Research &amp; Development</t>
+  </si>
+  <si>
+    <t>Sales</t>
+  </si>
+  <si>
+    <t>学历</t>
+  </si>
+  <si>
     <t>Education</t>
   </si>
   <si>
+    <t>专业</t>
+  </si>
+  <si>
     <t>EducationField</t>
   </si>
   <si>
+    <t>Computer Science</t>
+  </si>
+  <si>
+    <t>Marketing</t>
+  </si>
+  <si>
+    <t>性别</t>
+  </si>
+  <si>
     <t>Gender</t>
   </si>
   <si>
+    <t>Male</t>
+  </si>
+  <si>
+    <t>Female</t>
+  </si>
+  <si>
+    <t>职级</t>
+  </si>
+  <si>
     <t>JobLevel</t>
   </si>
   <si>
+    <t>岗位</t>
+  </si>
+  <si>
     <t>JobRole</t>
   </si>
   <si>
+    <t>Research Scientist</t>
+  </si>
+  <si>
+    <t>Sales Executive</t>
+  </si>
+  <si>
+    <t>婚姻</t>
+  </si>
+  <si>
     <t>MaritalStatus</t>
   </si>
   <si>
+    <t>Married</t>
+  </si>
+  <si>
+    <t>Single</t>
+  </si>
+  <si>
+    <t>月薪(元)</t>
+  </si>
+  <si>
     <t>MonthlyIncome</t>
   </si>
   <si>
+    <t>常加班?</t>
+  </si>
+  <si>
     <t>OverTime</t>
   </si>
   <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>涨薪%</t>
+  </si>
+  <si>
     <t>PercentSalaryHike</t>
   </si>
   <si>
+    <t>绩效</t>
+  </si>
+  <si>
     <t>PerformanceRating</t>
   </si>
   <si>
+    <t>总工龄</t>
+  </si>
+  <si>
     <t>TotalWorkingYears</t>
   </si>
   <si>
+    <t>本公司工龄</t>
+  </si>
+  <si>
     <t>YearsAtCompany</t>
   </si>
   <si>
+    <t>现岗年限</t>
+  </si>
+  <si>
     <t>YearsInCurrentRole</t>
   </si>
   <si>
+    <t>距晋升年数</t>
+  </si>
+  <si>
     <t>YearsSinceLastPromotion</t>
-  </si>
-  <si>
-    <t>No</t>
-  </si>
-  <si>
-    <t>Travel_Frequently</t>
-  </si>
-  <si>
-    <t>Travel_Rarely</t>
-  </si>
-  <si>
-    <t>Research &amp; Development</t>
-  </si>
-  <si>
-    <t>Sales</t>
-  </si>
-  <si>
-    <t>Computer Science</t>
-  </si>
-  <si>
-    <t>Marketing</t>
-  </si>
-  <si>
-    <t>Male</t>
-  </si>
-  <si>
-    <t>Female</t>
-  </si>
-  <si>
-    <t>Research Scientist</t>
-  </si>
-  <si>
-    <t>Sales Executive</t>
-  </si>
-  <si>
-    <t>Married</t>
-  </si>
-  <si>
-    <t>Single</t>
-  </si>
-  <si>
-    <t>Yes</t>
   </si>
 </sst>
 </file>
@@ -441,7 +495,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R3"/>
+  <dimension ref="A1:R4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
@@ -449,166 +503,222 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C1" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D1" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="E1" t="s">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="F1" t="s">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="G1" t="s">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="H1" t="s">
-        <v>7</v>
+        <v>23</v>
       </c>
       <c r="I1" t="s">
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="J1" t="s">
-        <v>9</v>
+        <v>29</v>
       </c>
       <c r="K1" t="s">
-        <v>10</v>
+        <v>33</v>
       </c>
       <c r="L1" t="s">
-        <v>11</v>
+        <v>35</v>
       </c>
       <c r="M1" t="s">
-        <v>12</v>
+        <v>38</v>
       </c>
       <c r="N1" t="s">
-        <v>13</v>
+        <v>40</v>
       </c>
       <c r="O1" t="s">
-        <v>14</v>
+        <v>42</v>
       </c>
       <c r="P1" t="s">
-        <v>15</v>
+        <v>44</v>
       </c>
       <c r="Q1" t="s">
-        <v>16</v>
+        <v>46</v>
       </c>
       <c r="R1" t="s">
-        <v>17</v>
+        <v>48</v>
       </c>
     </row>
     <row r="2" spans="1:18">
-      <c r="A2">
-        <v>35</v>
+      <c r="A2" t="s">
+        <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>18</v>
+        <v>3</v>
       </c>
       <c r="C2" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="D2" t="s">
-        <v>21</v>
-      </c>
-      <c r="E2">
-        <v>4</v>
+        <v>10</v>
+      </c>
+      <c r="E2" t="s">
+        <v>14</v>
       </c>
       <c r="F2" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="G2" t="s">
-        <v>25</v>
-      </c>
-      <c r="H2">
-        <v>3</v>
+        <v>20</v>
+      </c>
+      <c r="H2" t="s">
+        <v>24</v>
       </c>
       <c r="I2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="J2" t="s">
-        <v>29</v>
-      </c>
-      <c r="K2">
-        <v>32000</v>
+        <v>30</v>
+      </c>
+      <c r="K2" t="s">
+        <v>34</v>
       </c>
       <c r="L2" t="s">
-        <v>18</v>
-      </c>
-      <c r="M2">
-        <v>15</v>
-      </c>
-      <c r="N2">
-        <v>4</v>
-      </c>
-      <c r="O2">
-        <v>12</v>
-      </c>
-      <c r="P2">
-        <v>6</v>
-      </c>
-      <c r="Q2">
-        <v>4</v>
-      </c>
-      <c r="R2">
-        <v>3</v>
+        <v>36</v>
+      </c>
+      <c r="M2" t="s">
+        <v>39</v>
+      </c>
+      <c r="N2" t="s">
+        <v>41</v>
+      </c>
+      <c r="O2" t="s">
+        <v>43</v>
+      </c>
+      <c r="P2" t="s">
+        <v>45</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>47</v>
+      </c>
+      <c r="R2" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="3" spans="1:18">
       <c r="A3">
+        <v>35</v>
+      </c>
+      <c r="B3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3">
+        <v>4</v>
+      </c>
+      <c r="F3" t="s">
+        <v>17</v>
+      </c>
+      <c r="G3" t="s">
+        <v>21</v>
+      </c>
+      <c r="H3">
+        <v>3</v>
+      </c>
+      <c r="I3" t="s">
+        <v>27</v>
+      </c>
+      <c r="J3" t="s">
+        <v>31</v>
+      </c>
+      <c r="K3">
+        <v>32000</v>
+      </c>
+      <c r="L3" t="s">
+        <v>4</v>
+      </c>
+      <c r="M3">
+        <v>15</v>
+      </c>
+      <c r="N3">
+        <v>4</v>
+      </c>
+      <c r="O3">
+        <v>12</v>
+      </c>
+      <c r="P3">
+        <v>6</v>
+      </c>
+      <c r="Q3">
+        <v>4</v>
+      </c>
+      <c r="R3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18">
+      <c r="A4">
         <v>28</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4">
+        <v>3</v>
+      </c>
+      <c r="F4" t="s">
         <v>18</v>
       </c>
-      <c r="C3" t="s">
-        <v>20</v>
-      </c>
-      <c r="D3" t="s">
+      <c r="G4" t="s">
         <v>22</v>
       </c>
-      <c r="E3">
+      <c r="H4">
+        <v>2</v>
+      </c>
+      <c r="I4" t="s">
+        <v>28</v>
+      </c>
+      <c r="J4" t="s">
+        <v>32</v>
+      </c>
+      <c r="K4">
+        <v>18000</v>
+      </c>
+      <c r="L4" t="s">
+        <v>37</v>
+      </c>
+      <c r="M4">
+        <v>10</v>
+      </c>
+      <c r="N4">
         <v>3</v>
       </c>
-      <c r="F3" t="s">
-        <v>24</v>
-      </c>
-      <c r="G3" t="s">
-        <v>26</v>
-      </c>
-      <c r="H3">
+      <c r="O4">
+        <v>5</v>
+      </c>
+      <c r="P4">
         <v>2</v>
       </c>
-      <c r="I3" t="s">
-        <v>28</v>
-      </c>
-      <c r="J3" t="s">
-        <v>30</v>
-      </c>
-      <c r="K3">
-        <v>18000</v>
-      </c>
-      <c r="L3" t="s">
-        <v>31</v>
-      </c>
-      <c r="M3">
-        <v>10</v>
-      </c>
-      <c r="N3">
-        <v>3</v>
-      </c>
-      <c r="O3">
-        <v>5</v>
-      </c>
-      <c r="P3">
-        <v>2</v>
-      </c>
-      <c r="Q3">
+      <c r="Q4">
         <v>1</v>
       </c>
-      <c r="R3">
+      <c r="R4">
         <v>1</v>
       </c>
     </row>

</xml_diff>